<commit_message>
feature:- Youth_prod.xlcx add one user
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Email</t>
   </si>
@@ -98,28 +98,10 @@
     <t>EldonTrantow@yopmail.com</t>
   </si>
   <si>
-    <t>JeramyWest@yopmail.com</t>
-  </si>
-  <si>
-    <t>AlexKoch@yopmail.com</t>
-  </si>
-  <si>
-    <t>KarrenBarton@yopmail.com</t>
-  </si>
-  <si>
-    <t>EddieArmstrong@yopmail.com</t>
-  </si>
-  <si>
-    <t>AgripinaBartoletti@yopmail.com</t>
-  </si>
-  <si>
-    <t>ClaraKassulke@yopmail.com</t>
-  </si>
-  <si>
-    <t>IluminadaParisianV@yopmail.com</t>
-  </si>
-  <si>
-    <t>ShanaSawayn@yopmail.com</t>
+    <t>VeolaConsidine@yopmail.com</t>
+  </si>
+  <si>
+    <t>YvoneBerge@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -1279,7 +1261,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1407,36 +1389,6 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="s" s="0">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s" s="0">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s" s="0">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s" s="0">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s" s="0">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s" s="0">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
feature :- added beta super admin
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>rohank90020@maildrop.cc</t>
   </si>
@@ -119,6 +119,24 @@
   </si>
   <si>
     <t>rohank90054@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90057@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90058@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90056@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90059@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90060@maildrop.cc</t>
+  </si>
+  <si>
+    <t>rohank90061@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -1528,7 +1546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1720,6 +1738,36 @@
         <v>34</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 500 question bank (en, hi, ta, te, mr) + Confirm Publish dialog fixed
- Question bank: 500 questions (100 each in 5 languages)
- Server validates 200 (en+hi have proper script text)
- ta/te/mr need native script text for full validation
- Confirm Publish dialog: clicks red Publish button inside dialog
- All 10 tests pass end-to-end
</commit_message>
<xml_diff>
--- a/resources/Youth_prod.xlsx
+++ b/resources/Youth_prod.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="32">
   <si>
     <t>Email</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>Sankalp Vihar Elite Youth Club</t>
+  </si>
+  <si>
+    <t>ceolahomenick@maildrop.cc</t>
   </si>
 </sst>
 </file>
@@ -150,7 +153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -216,6 +219,11 @@
     <row r="13">
       <c r="A13" t="s" s="0">
         <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>